<commit_message>
Score the blind spot-check and update docs with the real result
Mean kappa 0.71 on the 8 topics with >=5 examples; churn_intent kappa 0.35,
traced to a definitional gap (warn-others vs explicit switch).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/labels/spotcheck_blind.xlsx
+++ b/data/labels/spotcheck_blind.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\non-tech\data\labels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD7EC3AD-698F-4E8E-BF40-DADA93A00630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BE3BBF9-D977-4269-B855-D469CA78E557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="265">
   <si>
     <t>review_id</t>
   </si>
@@ -812,6 +812,9 @@
   </si>
   <si>
     <t>phone pay</t>
+  </si>
+  <si>
+    <t>google pay</t>
   </si>
 </sst>
 </file>
@@ -1185,7 +1188,7 @@
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="3" max="3" width="7.21875" customWidth="1"/>
     <col min="4" max="4" width="70" customWidth="1"/>
     <col min="5" max="23" width="15" customWidth="1"/>
     <col min="24" max="24" width="14" customWidth="1"/>
@@ -2891,7 +2894,9 @@
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
-      <c r="J46" s="2"/>
+      <c r="J46" s="2">
+        <v>1</v>
+      </c>
       <c r="K46" s="2"/>
       <c r="L46" s="2"/>
       <c r="M46" s="2"/>
@@ -2936,7 +2941,9 @@
       <c r="R47" s="2"/>
       <c r="S47" s="2"/>
       <c r="T47" s="2"/>
-      <c r="U47" s="2"/>
+      <c r="U47" s="2">
+        <v>1</v>
+      </c>
       <c r="V47" s="2"/>
       <c r="W47" s="2"/>
       <c r="X47" s="2"/>
@@ -2960,8 +2967,12 @@
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
-      <c r="K48" s="2"/>
-      <c r="L48" s="2"/>
+      <c r="K48" s="2">
+        <v>1</v>
+      </c>
+      <c r="L48" s="2">
+        <v>1</v>
+      </c>
       <c r="M48" s="2"/>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
@@ -3004,7 +3015,9 @@
       <c r="R49" s="2"/>
       <c r="S49" s="2"/>
       <c r="T49" s="2"/>
-      <c r="U49" s="2"/>
+      <c r="U49" s="2">
+        <v>1</v>
+      </c>
       <c r="V49" s="2"/>
       <c r="W49" s="2"/>
       <c r="X49" s="2"/>
@@ -3028,7 +3041,9 @@
       <c r="H50" s="2"/>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
-      <c r="K50" s="2"/>
+      <c r="K50" s="2">
+        <v>1</v>
+      </c>
       <c r="L50" s="2"/>
       <c r="M50" s="2"/>
       <c r="N50" s="2"/>
@@ -3041,7 +3056,9 @@
       <c r="U50" s="2"/>
       <c r="V50" s="2"/>
       <c r="W50" s="2"/>
-      <c r="X50" s="2"/>
+      <c r="X50" s="2" t="s">
+        <v>264</v>
+      </c>
     </row>
     <row r="51" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
@@ -3065,14 +3082,18 @@
       <c r="K51" s="2"/>
       <c r="L51" s="2"/>
       <c r="M51" s="2"/>
-      <c r="N51" s="2"/>
+      <c r="N51" s="2">
+        <v>1</v>
+      </c>
       <c r="O51" s="2"/>
       <c r="P51" s="2"/>
       <c r="Q51" s="2"/>
       <c r="R51" s="2"/>
       <c r="S51" s="2"/>
       <c r="T51" s="2"/>
-      <c r="U51" s="2"/>
+      <c r="U51" s="2">
+        <v>1</v>
+      </c>
       <c r="V51" s="2"/>
       <c r="W51" s="2"/>
       <c r="X51" s="2"/>
@@ -3106,7 +3127,9 @@
       <c r="R52" s="2"/>
       <c r="S52" s="2"/>
       <c r="T52" s="2"/>
-      <c r="U52" s="2"/>
+      <c r="U52" s="2">
+        <v>1</v>
+      </c>
       <c r="V52" s="2"/>
       <c r="W52" s="2"/>
       <c r="X52" s="2"/>
@@ -3127,7 +3150,9 @@
       <c r="E53" s="2"/>
       <c r="F53" s="2"/>
       <c r="G53" s="2"/>
-      <c r="H53" s="2"/>
+      <c r="H53" s="2">
+        <v>1</v>
+      </c>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
       <c r="K53" s="2"/>
@@ -3174,7 +3199,9 @@
       <c r="R54" s="2"/>
       <c r="S54" s="2"/>
       <c r="T54" s="2"/>
-      <c r="U54" s="2"/>
+      <c r="U54" s="2">
+        <v>1</v>
+      </c>
       <c r="V54" s="2"/>
       <c r="W54" s="2"/>
       <c r="X54" s="2"/>
@@ -3192,14 +3219,18 @@
       <c r="D55" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="E55" s="2"/>
+      <c r="E55" s="2">
+        <v>1</v>
+      </c>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
-      <c r="L55" s="2"/>
+      <c r="L55" s="2">
+        <v>1</v>
+      </c>
       <c r="M55" s="2"/>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -3230,7 +3261,9 @@
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
-      <c r="I56" s="2"/>
+      <c r="I56" s="2">
+        <v>1</v>
+      </c>
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
       <c r="L56" s="2"/>
@@ -3265,7 +3298,9 @@
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
-      <c r="J57" s="2"/>
+      <c r="J57" s="2">
+        <v>1</v>
+      </c>
       <c r="K57" s="2"/>
       <c r="L57" s="2"/>
       <c r="M57" s="2"/>
@@ -3310,10 +3345,14 @@
       <c r="R58" s="2"/>
       <c r="S58" s="2"/>
       <c r="T58" s="2"/>
-      <c r="U58" s="2"/>
+      <c r="U58" s="2">
+        <v>1</v>
+      </c>
       <c r="V58" s="2"/>
       <c r="W58" s="2"/>
-      <c r="X58" s="2"/>
+      <c r="X58" s="2" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="59" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
@@ -3367,7 +3406,9 @@
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
       <c r="I60" s="2"/>
-      <c r="J60" s="2"/>
+      <c r="J60" s="2">
+        <v>1</v>
+      </c>
       <c r="K60" s="2"/>
       <c r="L60" s="2"/>
       <c r="M60" s="2"/>
@@ -3412,7 +3453,9 @@
       <c r="R61" s="2"/>
       <c r="S61" s="2"/>
       <c r="T61" s="2"/>
-      <c r="U61" s="2"/>
+      <c r="U61" s="2">
+        <v>1</v>
+      </c>
       <c r="V61" s="2"/>
       <c r="W61" s="2"/>
       <c r="X61" s="2"/>
@@ -3447,7 +3490,9 @@
       <c r="S62" s="2"/>
       <c r="T62" s="2"/>
       <c r="U62" s="2"/>
-      <c r="V62" s="2"/>
+      <c r="V62" s="2">
+        <v>1</v>
+      </c>
       <c r="W62" s="2"/>
       <c r="X62" s="2"/>
     </row>
@@ -3473,10 +3518,16 @@
       <c r="K63" s="2"/>
       <c r="L63" s="2"/>
       <c r="M63" s="2"/>
-      <c r="N63" s="2"/>
-      <c r="O63" s="2"/>
+      <c r="N63" s="2">
+        <v>1</v>
+      </c>
+      <c r="O63" s="2">
+        <v>1</v>
+      </c>
       <c r="P63" s="2"/>
-      <c r="Q63" s="2"/>
+      <c r="Q63" s="2">
+        <v>1</v>
+      </c>
       <c r="R63" s="2"/>
       <c r="S63" s="2"/>
       <c r="T63" s="2"/>
@@ -3503,15 +3554,21 @@
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
-      <c r="J64" s="2"/>
+      <c r="J64" s="2">
+        <v>1</v>
+      </c>
       <c r="K64" s="2"/>
-      <c r="L64" s="2"/>
+      <c r="L64" s="2">
+        <v>1</v>
+      </c>
       <c r="M64" s="2"/>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
       <c r="P64" s="2"/>
       <c r="Q64" s="2"/>
-      <c r="R64" s="2"/>
+      <c r="R64" s="2">
+        <v>1</v>
+      </c>
       <c r="S64" s="2"/>
       <c r="T64" s="2"/>
       <c r="U64" s="2"/>
@@ -3537,7 +3594,9 @@
       <c r="G65" s="2"/>
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
-      <c r="J65" s="2"/>
+      <c r="J65" s="2">
+        <v>1</v>
+      </c>
       <c r="K65" s="2"/>
       <c r="L65" s="2"/>
       <c r="M65" s="2"/>
@@ -3571,8 +3630,12 @@
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
       <c r="I66" s="2"/>
-      <c r="J66" s="2"/>
-      <c r="K66" s="2"/>
+      <c r="J66" s="2">
+        <v>1</v>
+      </c>
+      <c r="K66" s="2">
+        <v>1</v>
+      </c>
       <c r="L66" s="2"/>
       <c r="M66" s="2"/>
       <c r="N66" s="2"/>
@@ -3617,7 +3680,9 @@
       <c r="S67" s="2"/>
       <c r="T67" s="2"/>
       <c r="U67" s="2"/>
-      <c r="V67" s="2"/>
+      <c r="V67" s="2">
+        <v>1</v>
+      </c>
       <c r="W67" s="2"/>
       <c r="X67" s="2"/>
     </row>
@@ -3643,7 +3708,9 @@
       <c r="K68" s="2"/>
       <c r="L68" s="2"/>
       <c r="M68" s="2"/>
-      <c r="N68" s="2"/>
+      <c r="N68" s="2">
+        <v>1</v>
+      </c>
       <c r="O68" s="2"/>
       <c r="P68" s="2"/>
       <c r="Q68" s="2"/>
@@ -3711,14 +3778,18 @@
       <c r="K70" s="2"/>
       <c r="L70" s="2"/>
       <c r="M70" s="2"/>
-      <c r="N70" s="2"/>
+      <c r="N70" s="2">
+        <v>1</v>
+      </c>
       <c r="O70" s="2"/>
       <c r="P70" s="2"/>
       <c r="Q70" s="2"/>
       <c r="R70" s="2"/>
       <c r="S70" s="2"/>
       <c r="T70" s="2"/>
-      <c r="U70" s="2"/>
+      <c r="U70" s="2">
+        <v>1</v>
+      </c>
       <c r="V70" s="2"/>
       <c r="W70" s="2"/>
       <c r="X70" s="2"/>
@@ -3753,7 +3824,9 @@
       <c r="S71" s="2"/>
       <c r="T71" s="2"/>
       <c r="U71" s="2"/>
-      <c r="V71" s="2"/>
+      <c r="V71" s="2">
+        <v>1</v>
+      </c>
       <c r="W71" s="2"/>
       <c r="X71" s="2"/>
     </row>
@@ -3770,7 +3843,9 @@
       <c r="D72" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="E72" s="2"/>
+      <c r="E72" s="2">
+        <v>1</v>
+      </c>
       <c r="F72" s="2"/>
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
@@ -3788,7 +3863,9 @@
       <c r="T72" s="2"/>
       <c r="U72" s="2"/>
       <c r="V72" s="2"/>
-      <c r="W72" s="2"/>
+      <c r="W72" s="2">
+        <v>1</v>
+      </c>
       <c r="X72" s="2"/>
     </row>
     <row r="73" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3804,14 +3881,18 @@
       <c r="D73" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="E73" s="2"/>
+      <c r="E73" s="2">
+        <v>1</v>
+      </c>
       <c r="F73" s="2"/>
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
       <c r="K73" s="2"/>
-      <c r="L73" s="2"/>
+      <c r="L73" s="2">
+        <v>1</v>
+      </c>
       <c r="M73" s="2"/>
       <c r="N73" s="2"/>
       <c r="O73" s="2"/>
@@ -3848,7 +3929,9 @@
       <c r="L74" s="2"/>
       <c r="M74" s="2"/>
       <c r="N74" s="2"/>
-      <c r="O74" s="2"/>
+      <c r="O74" s="2">
+        <v>1</v>
+      </c>
       <c r="P74" s="2"/>
       <c r="Q74" s="2"/>
       <c r="R74" s="2"/>
@@ -3856,7 +3939,9 @@
       <c r="T74" s="2"/>
       <c r="U74" s="2"/>
       <c r="V74" s="2"/>
-      <c r="W74" s="2"/>
+      <c r="W74" s="2">
+        <v>1</v>
+      </c>
       <c r="X74" s="2"/>
     </row>
     <row r="75" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3872,7 +3957,9 @@
       <c r="D75" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="E75" s="2"/>
+      <c r="E75" s="2">
+        <v>1</v>
+      </c>
       <c r="F75" s="2"/>
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
@@ -3922,7 +4009,9 @@
       <c r="R76" s="2"/>
       <c r="S76" s="2"/>
       <c r="T76" s="2"/>
-      <c r="U76" s="2"/>
+      <c r="U76" s="2">
+        <v>1</v>
+      </c>
       <c r="V76" s="2"/>
       <c r="W76" s="2"/>
       <c r="X76" s="2"/>
@@ -3956,7 +4045,9 @@
       <c r="R77" s="2"/>
       <c r="S77" s="2"/>
       <c r="T77" s="2"/>
-      <c r="U77" s="2"/>
+      <c r="U77" s="2">
+        <v>1</v>
+      </c>
       <c r="V77" s="2"/>
       <c r="W77" s="2"/>
       <c r="X77" s="2"/>
@@ -3983,7 +4074,9 @@
       <c r="K78" s="2"/>
       <c r="L78" s="2"/>
       <c r="M78" s="2"/>
-      <c r="N78" s="2"/>
+      <c r="N78" s="2">
+        <v>1</v>
+      </c>
       <c r="O78" s="2"/>
       <c r="P78" s="2"/>
       <c r="Q78" s="2"/>
@@ -4008,7 +4101,9 @@
       <c r="D79" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="E79" s="2"/>
+      <c r="E79" s="2">
+        <v>1</v>
+      </c>
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
@@ -4059,7 +4154,9 @@
       <c r="S80" s="2"/>
       <c r="T80" s="2"/>
       <c r="U80" s="2"/>
-      <c r="V80" s="2"/>
+      <c r="V80" s="2">
+        <v>1</v>
+      </c>
       <c r="W80" s="2"/>
       <c r="X80" s="2"/>
     </row>
@@ -4088,9 +4185,13 @@
       <c r="N81" s="2"/>
       <c r="O81" s="2"/>
       <c r="P81" s="2"/>
-      <c r="Q81" s="2"/>
+      <c r="Q81" s="2">
+        <v>1</v>
+      </c>
       <c r="R81" s="2"/>
-      <c r="S81" s="2"/>
+      <c r="S81" s="2">
+        <v>1</v>
+      </c>
       <c r="T81" s="2"/>
       <c r="U81" s="2"/>
       <c r="V81" s="2"/>
@@ -4126,7 +4227,9 @@
       <c r="R82" s="2"/>
       <c r="S82" s="2"/>
       <c r="T82" s="2"/>
-      <c r="U82" s="2"/>
+      <c r="U82" s="2">
+        <v>1</v>
+      </c>
       <c r="V82" s="2"/>
       <c r="W82" s="2"/>
       <c r="X82" s="2"/>
@@ -4160,7 +4263,9 @@
       <c r="R83" s="2"/>
       <c r="S83" s="2"/>
       <c r="T83" s="2"/>
-      <c r="U83" s="2"/>
+      <c r="U83" s="2">
+        <v>1</v>
+      </c>
       <c r="V83" s="2"/>
       <c r="W83" s="2"/>
       <c r="X83" s="2"/>
@@ -4187,7 +4292,9 @@
       <c r="K84" s="2"/>
       <c r="L84" s="2"/>
       <c r="M84" s="2"/>
-      <c r="N84" s="2"/>
+      <c r="N84" s="2">
+        <v>1</v>
+      </c>
       <c r="O84" s="2"/>
       <c r="P84" s="2"/>
       <c r="Q84" s="2"/>
@@ -4228,7 +4335,9 @@
       <c r="R85" s="2"/>
       <c r="S85" s="2"/>
       <c r="T85" s="2"/>
-      <c r="U85" s="2"/>
+      <c r="U85" s="2">
+        <v>1</v>
+      </c>
       <c r="V85" s="2"/>
       <c r="W85" s="2"/>
       <c r="X85" s="2"/>
@@ -4258,11 +4367,15 @@
       <c r="N86" s="2"/>
       <c r="O86" s="2"/>
       <c r="P86" s="2"/>
-      <c r="Q86" s="2"/>
+      <c r="Q86" s="2">
+        <v>1</v>
+      </c>
       <c r="R86" s="2"/>
       <c r="S86" s="2"/>
       <c r="T86" s="2"/>
-      <c r="U86" s="2"/>
+      <c r="U86" s="2">
+        <v>1</v>
+      </c>
       <c r="V86" s="2"/>
       <c r="W86" s="2"/>
       <c r="X86" s="2"/>
@@ -4287,7 +4400,9 @@
       <c r="I87" s="2"/>
       <c r="J87" s="2"/>
       <c r="K87" s="2"/>
-      <c r="L87" s="2"/>
+      <c r="L87" s="2">
+        <v>1</v>
+      </c>
       <c r="M87" s="2"/>
       <c r="N87" s="2"/>
       <c r="O87" s="2"/>
@@ -4330,7 +4445,9 @@
       <c r="R88" s="2"/>
       <c r="S88" s="2"/>
       <c r="T88" s="2"/>
-      <c r="U88" s="2"/>
+      <c r="U88" s="2">
+        <v>1</v>
+      </c>
       <c r="V88" s="2"/>
       <c r="W88" s="2"/>
       <c r="X88" s="2"/>
@@ -4364,7 +4481,9 @@
       <c r="R89" s="2"/>
       <c r="S89" s="2"/>
       <c r="T89" s="2"/>
-      <c r="U89" s="2"/>
+      <c r="U89" s="2">
+        <v>1</v>
+      </c>
       <c r="V89" s="2"/>
       <c r="W89" s="2"/>
       <c r="X89" s="2"/>
@@ -4398,7 +4517,9 @@
       <c r="R90" s="2"/>
       <c r="S90" s="2"/>
       <c r="T90" s="2"/>
-      <c r="U90" s="2"/>
+      <c r="U90" s="2">
+        <v>1</v>
+      </c>
       <c r="V90" s="2"/>
       <c r="W90" s="2"/>
       <c r="X90" s="2"/>
@@ -4432,7 +4553,9 @@
       <c r="R91" s="2"/>
       <c r="S91" s="2"/>
       <c r="T91" s="2"/>
-      <c r="U91" s="2"/>
+      <c r="U91" s="2">
+        <v>1</v>
+      </c>
       <c r="V91" s="2"/>
       <c r="W91" s="2"/>
       <c r="X91" s="2"/>
@@ -4466,7 +4589,9 @@
       <c r="R92" s="2"/>
       <c r="S92" s="2"/>
       <c r="T92" s="2"/>
-      <c r="U92" s="2"/>
+      <c r="U92" s="2">
+        <v>1</v>
+      </c>
       <c r="V92" s="2"/>
       <c r="W92" s="2"/>
       <c r="X92" s="2"/>
@@ -4489,9 +4614,13 @@
       <c r="G93" s="2"/>
       <c r="H93" s="2"/>
       <c r="I93" s="2"/>
-      <c r="J93" s="2"/>
+      <c r="J93" s="2">
+        <v>1</v>
+      </c>
       <c r="K93" s="2"/>
-      <c r="L93" s="2"/>
+      <c r="L93" s="2">
+        <v>1</v>
+      </c>
       <c r="M93" s="2"/>
       <c r="N93" s="2"/>
       <c r="O93" s="2"/>
@@ -4534,7 +4663,9 @@
       <c r="R94" s="2"/>
       <c r="S94" s="2"/>
       <c r="T94" s="2"/>
-      <c r="U94" s="2"/>
+      <c r="U94" s="2">
+        <v>1</v>
+      </c>
       <c r="V94" s="2"/>
       <c r="W94" s="2"/>
       <c r="X94" s="2"/>
@@ -4559,7 +4690,9 @@
       <c r="I95" s="2"/>
       <c r="J95" s="2"/>
       <c r="K95" s="2"/>
-      <c r="L95" s="2"/>
+      <c r="L95" s="2">
+        <v>1</v>
+      </c>
       <c r="M95" s="2"/>
       <c r="N95" s="2"/>
       <c r="O95" s="2"/>
@@ -4599,12 +4732,16 @@
       <c r="O96" s="2"/>
       <c r="P96" s="2"/>
       <c r="Q96" s="2"/>
-      <c r="R96" s="2"/>
+      <c r="R96" s="2">
+        <v>1</v>
+      </c>
       <c r="S96" s="2"/>
       <c r="T96" s="2"/>
       <c r="U96" s="2"/>
       <c r="V96" s="2"/>
-      <c r="W96" s="2"/>
+      <c r="W96" s="2">
+        <v>1</v>
+      </c>
       <c r="X96" s="2"/>
     </row>
     <row r="97" spans="1:24" ht="120" customHeight="1" x14ac:dyDescent="0.3">
@@ -4628,7 +4765,9 @@
       <c r="J97" s="2"/>
       <c r="K97" s="2"/>
       <c r="L97" s="2"/>
-      <c r="M97" s="2"/>
+      <c r="M97" s="2">
+        <v>1</v>
+      </c>
       <c r="N97" s="2"/>
       <c r="O97" s="2"/>
       <c r="P97" s="2"/>
@@ -4638,7 +4777,9 @@
       <c r="T97" s="2"/>
       <c r="U97" s="2"/>
       <c r="V97" s="2"/>
-      <c r="W97" s="2"/>
+      <c r="W97" s="2">
+        <v>1</v>
+      </c>
       <c r="X97" s="2"/>
     </row>
     <row r="98" spans="1:24" ht="75" customHeight="1" x14ac:dyDescent="0.3">
@@ -4654,14 +4795,18 @@
       <c r="D98" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="E98" s="2"/>
+      <c r="E98" s="2">
+        <v>1</v>
+      </c>
       <c r="F98" s="2"/>
       <c r="G98" s="2"/>
       <c r="H98" s="2"/>
       <c r="I98" s="2"/>
       <c r="J98" s="2"/>
       <c r="K98" s="2"/>
-      <c r="L98" s="2"/>
+      <c r="L98" s="2">
+        <v>1</v>
+      </c>
       <c r="M98" s="2"/>
       <c r="N98" s="2"/>
       <c r="O98" s="2"/>
@@ -4672,7 +4817,9 @@
       <c r="T98" s="2"/>
       <c r="U98" s="2"/>
       <c r="V98" s="2"/>
-      <c r="W98" s="2"/>
+      <c r="W98" s="2">
+        <v>1</v>
+      </c>
       <c r="X98" s="2"/>
     </row>
     <row r="99" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -4693,7 +4840,9 @@
       <c r="G99" s="2"/>
       <c r="H99" s="2"/>
       <c r="I99" s="2"/>
-      <c r="J99" s="2"/>
+      <c r="J99" s="2">
+        <v>1</v>
+      </c>
       <c r="K99" s="2"/>
       <c r="L99" s="2"/>
       <c r="M99" s="2"/>
@@ -4730,8 +4879,12 @@
       <c r="J100" s="2"/>
       <c r="K100" s="2"/>
       <c r="L100" s="2"/>
-      <c r="M100" s="2"/>
-      <c r="N100" s="2"/>
+      <c r="M100" s="2">
+        <v>1</v>
+      </c>
+      <c r="N100" s="2">
+        <v>1</v>
+      </c>
       <c r="O100" s="2"/>
       <c r="P100" s="2"/>
       <c r="Q100" s="2"/>
@@ -4772,7 +4925,9 @@
       <c r="R101" s="2"/>
       <c r="S101" s="2"/>
       <c r="T101" s="2"/>
-      <c r="U101" s="2"/>
+      <c r="U101" s="2">
+        <v>1</v>
+      </c>
       <c r="V101" s="2"/>
       <c r="W101" s="2"/>
       <c r="X101" s="2"/>
@@ -4795,14 +4950,20 @@
       <c r="G102" s="2"/>
       <c r="H102" s="2"/>
       <c r="I102" s="2"/>
-      <c r="J102" s="2"/>
-      <c r="K102" s="2"/>
+      <c r="J102" s="2">
+        <v>1</v>
+      </c>
+      <c r="K102" s="2">
+        <v>1</v>
+      </c>
       <c r="L102" s="2"/>
       <c r="M102" s="2"/>
       <c r="N102" s="2"/>
       <c r="O102" s="2"/>
       <c r="P102" s="2"/>
-      <c r="Q102" s="2"/>
+      <c r="Q102" s="2">
+        <v>1</v>
+      </c>
       <c r="R102" s="2"/>
       <c r="S102" s="2"/>
       <c r="T102" s="2"/>
@@ -4840,7 +5001,9 @@
       <c r="R103" s="2"/>
       <c r="S103" s="2"/>
       <c r="T103" s="2"/>
-      <c r="U103" s="2"/>
+      <c r="U103" s="2">
+        <v>1</v>
+      </c>
       <c r="V103" s="2"/>
       <c r="W103" s="2"/>
       <c r="X103" s="2"/>
@@ -4874,7 +5037,9 @@
       <c r="R104" s="2"/>
       <c r="S104" s="2"/>
       <c r="T104" s="2"/>
-      <c r="U104" s="2"/>
+      <c r="U104" s="2">
+        <v>1</v>
+      </c>
       <c r="V104" s="2"/>
       <c r="W104" s="2"/>
       <c r="X104" s="2"/>
@@ -4908,7 +5073,9 @@
       <c r="R105" s="2"/>
       <c r="S105" s="2"/>
       <c r="T105" s="2"/>
-      <c r="U105" s="2"/>
+      <c r="U105" s="2">
+        <v>1</v>
+      </c>
       <c r="V105" s="2"/>
       <c r="W105" s="2"/>
       <c r="X105" s="2"/>
@@ -4932,7 +5099,9 @@
       <c r="H106" s="2"/>
       <c r="I106" s="2"/>
       <c r="J106" s="2"/>
-      <c r="K106" s="2"/>
+      <c r="K106" s="2">
+        <v>1</v>
+      </c>
       <c r="L106" s="2"/>
       <c r="M106" s="2"/>
       <c r="N106" s="2"/>
@@ -4965,7 +5134,9 @@
       <c r="G107" s="2"/>
       <c r="H107" s="2"/>
       <c r="I107" s="2"/>
-      <c r="J107" s="2"/>
+      <c r="J107" s="2">
+        <v>1</v>
+      </c>
       <c r="K107" s="2"/>
       <c r="L107" s="2"/>
       <c r="M107" s="2"/>
@@ -4999,7 +5170,9 @@
       <c r="G108" s="2"/>
       <c r="H108" s="2"/>
       <c r="I108" s="2"/>
-      <c r="J108" s="2"/>
+      <c r="J108" s="2">
+        <v>1</v>
+      </c>
       <c r="K108" s="2"/>
       <c r="L108" s="2"/>
       <c r="M108" s="2"/>
@@ -5038,7 +5211,9 @@
       <c r="L109" s="2"/>
       <c r="M109" s="2"/>
       <c r="N109" s="2"/>
-      <c r="O109" s="2"/>
+      <c r="O109" s="2">
+        <v>1</v>
+      </c>
       <c r="P109" s="2"/>
       <c r="Q109" s="2"/>
       <c r="R109" s="2"/>
@@ -5067,9 +5242,13 @@
       <c r="G110" s="2"/>
       <c r="H110" s="2"/>
       <c r="I110" s="2"/>
-      <c r="J110" s="2"/>
+      <c r="J110" s="2">
+        <v>1</v>
+      </c>
       <c r="K110" s="2"/>
-      <c r="L110" s="2"/>
+      <c r="L110" s="2">
+        <v>1</v>
+      </c>
       <c r="M110" s="2"/>
       <c r="N110" s="2"/>
       <c r="O110" s="2"/>
@@ -5101,7 +5280,9 @@
       <c r="G111" s="2"/>
       <c r="H111" s="2"/>
       <c r="I111" s="2"/>
-      <c r="J111" s="2"/>
+      <c r="J111" s="2">
+        <v>1</v>
+      </c>
       <c r="K111" s="2"/>
       <c r="L111" s="2"/>
       <c r="M111" s="2"/>
@@ -5130,13 +5311,17 @@
       <c r="D112" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="E112" s="2"/>
+      <c r="E112" s="2">
+        <v>1</v>
+      </c>
       <c r="F112" s="2"/>
       <c r="G112" s="2"/>
       <c r="H112" s="2"/>
       <c r="I112" s="2"/>
       <c r="J112" s="2"/>
-      <c r="K112" s="2"/>
+      <c r="K112" s="2">
+        <v>1</v>
+      </c>
       <c r="L112" s="2"/>
       <c r="M112" s="2"/>
       <c r="N112" s="2"/>
@@ -5170,7 +5355,9 @@
       <c r="H113" s="2"/>
       <c r="I113" s="2"/>
       <c r="J113" s="2"/>
-      <c r="K113" s="2"/>
+      <c r="K113" s="2">
+        <v>1</v>
+      </c>
       <c r="L113" s="2"/>
       <c r="M113" s="2"/>
       <c r="N113" s="2"/>
@@ -5180,7 +5367,9 @@
       <c r="R113" s="2"/>
       <c r="S113" s="2"/>
       <c r="T113" s="2"/>
-      <c r="U113" s="2"/>
+      <c r="U113" s="2">
+        <v>1</v>
+      </c>
       <c r="V113" s="2"/>
       <c r="W113" s="2"/>
       <c r="X113" s="2"/>
@@ -5205,7 +5394,9 @@
       <c r="I114" s="2"/>
       <c r="J114" s="2"/>
       <c r="K114" s="2"/>
-      <c r="L114" s="2"/>
+      <c r="L114" s="2">
+        <v>1</v>
+      </c>
       <c r="M114" s="2"/>
       <c r="N114" s="2"/>
       <c r="O114" s="2"/>
@@ -5238,7 +5429,9 @@
       <c r="H115" s="2"/>
       <c r="I115" s="2"/>
       <c r="J115" s="2"/>
-      <c r="K115" s="2"/>
+      <c r="K115" s="2">
+        <v>1</v>
+      </c>
       <c r="L115" s="2"/>
       <c r="M115" s="2"/>
       <c r="N115" s="2"/>
@@ -5268,9 +5461,13 @@
       </c>
       <c r="E116" s="2"/>
       <c r="F116" s="2"/>
-      <c r="G116" s="2"/>
+      <c r="G116" s="2">
+        <v>1</v>
+      </c>
       <c r="H116" s="2"/>
-      <c r="I116" s="2"/>
+      <c r="I116" s="2">
+        <v>1</v>
+      </c>
       <c r="J116" s="2"/>
       <c r="K116" s="2"/>
       <c r="L116" s="2"/>
@@ -5306,7 +5503,9 @@
       <c r="H117" s="2"/>
       <c r="I117" s="2"/>
       <c r="J117" s="2"/>
-      <c r="K117" s="2"/>
+      <c r="K117" s="2">
+        <v>1</v>
+      </c>
       <c r="L117" s="2"/>
       <c r="M117" s="2"/>
       <c r="N117" s="2"/>
@@ -5373,7 +5572,9 @@
       <c r="G119" s="2"/>
       <c r="H119" s="2"/>
       <c r="I119" s="2"/>
-      <c r="J119" s="2"/>
+      <c r="J119" s="2">
+        <v>1</v>
+      </c>
       <c r="K119" s="2"/>
       <c r="L119" s="2"/>
       <c r="M119" s="2"/>
@@ -5411,7 +5612,9 @@
       <c r="K120" s="2"/>
       <c r="L120" s="2"/>
       <c r="M120" s="2"/>
-      <c r="N120" s="2"/>
+      <c r="N120" s="2">
+        <v>1</v>
+      </c>
       <c r="O120" s="2"/>
       <c r="P120" s="2"/>
       <c r="Q120" s="2"/>
@@ -5420,7 +5623,9 @@
       <c r="T120" s="2"/>
       <c r="U120" s="2"/>
       <c r="V120" s="2"/>
-      <c r="W120" s="2"/>
+      <c r="W120" s="2">
+        <v>1</v>
+      </c>
       <c r="X120" s="2"/>
     </row>
     <row r="121" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -5452,7 +5657,9 @@
       <c r="R121" s="2"/>
       <c r="S121" s="2"/>
       <c r="T121" s="2"/>
-      <c r="U121" s="2"/>
+      <c r="U121" s="2">
+        <v>1</v>
+      </c>
       <c r="V121" s="2"/>
       <c r="W121" s="2"/>
       <c r="X121" s="2"/>

</xml_diff>

<commit_message>
Apply adjudicated third pass of spot-check label edits
14 edits checked against review text; reported as optimistic since made
after seeing disagreements. First-pass score remains the headline.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/labels/spotcheck_blind.xlsx
+++ b/data/labels/spotcheck_blind.xlsx
@@ -686,7 +686,11 @@
       <c r="E4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="2" t="n"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
@@ -792,9 +796,7 @@
       <c r="S6" s="2" t="n"/>
       <c r="T6" s="2" t="n"/>
       <c r="U6" s="2" t="n"/>
-      <c r="V6" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="V6" s="2" t="n"/>
       <c r="W6" s="2" t="n"/>
       <c r="X6" s="2" t="n"/>
     </row>
@@ -841,9 +843,7 @@
       <c r="T7" s="2" t="n"/>
       <c r="U7" s="2" t="n"/>
       <c r="V7" s="2" t="n"/>
-      <c r="W7" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="W7" s="2" t="n"/>
       <c r="X7" s="2" t="inlineStr">
         <is>
           <t>bhim</t>
@@ -1022,9 +1022,7 @@
       <c r="S11" s="2" t="n"/>
       <c r="T11" s="2" t="n"/>
       <c r="U11" s="2" t="n"/>
-      <c r="V11" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="V11" s="2" t="n"/>
       <c r="W11" s="2" t="n"/>
       <c r="X11" s="2" t="n"/>
     </row>
@@ -2269,9 +2267,7 @@
       <c r="T39" s="2" t="n"/>
       <c r="U39" s="2" t="n"/>
       <c r="V39" s="2" t="n"/>
-      <c r="W39" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="W39" s="2" t="n"/>
       <c r="X39" s="2" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1">
@@ -2447,9 +2443,7 @@
       <c r="V43" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="W43" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="W43" s="2" t="n"/>
       <c r="X43" s="2" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1">
@@ -2966,7 +2960,11 @@
       <c r="E55" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F55" s="2" t="n"/>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="G55" s="2" t="n"/>
       <c r="H55" s="2" t="n"/>
       <c r="I55" s="2" t="n"/>
@@ -3118,11 +3116,7 @@
       </c>
       <c r="V58" s="2" t="n"/>
       <c r="W58" s="2" t="n"/>
-      <c r="X58" s="2" t="inlineStr">
-        <is>
-          <t>phonepe</t>
-        </is>
-      </c>
+      <c r="X58" s="2" t="n"/>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
@@ -3751,9 +3745,7 @@
       <c r="T72" s="2" t="n"/>
       <c r="U72" s="2" t="n"/>
       <c r="V72" s="2" t="n"/>
-      <c r="W72" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="W72" s="2" t="n"/>
       <c r="X72" s="2" t="n"/>
     </row>
     <row r="73" ht="30" customHeight="1">
@@ -3843,9 +3835,7 @@
       <c r="T74" s="2" t="n"/>
       <c r="U74" s="2" t="n"/>
       <c r="V74" s="2" t="n"/>
-      <c r="W74" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="W74" s="2" t="n"/>
       <c r="X74" s="2" t="n"/>
     </row>
     <row r="75" ht="30" customHeight="1">
@@ -4817,9 +4807,7 @@
       <c r="T96" s="2" t="n"/>
       <c r="U96" s="2" t="n"/>
       <c r="V96" s="2" t="n"/>
-      <c r="W96" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="W96" s="2" t="n"/>
       <c r="X96" s="2" t="n"/>
     </row>
     <row r="97" ht="120" customHeight="1">
@@ -4845,7 +4833,11 @@
       </c>
       <c r="E97" s="2" t="n"/>
       <c r="F97" s="2" t="n"/>
-      <c r="G97" s="2" t="n"/>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="H97" s="2" t="n"/>
       <c r="I97" s="2" t="n"/>
       <c r="J97" s="2" t="n"/>
@@ -4863,9 +4855,7 @@
       <c r="T97" s="2" t="n"/>
       <c r="U97" s="2" t="n"/>
       <c r="V97" s="2" t="n"/>
-      <c r="W97" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="W97" s="2" t="n"/>
       <c r="X97" s="2" t="n"/>
     </row>
     <row r="98" ht="75" customHeight="1">
@@ -4911,9 +4901,7 @@
       <c r="T98" s="2" t="n"/>
       <c r="U98" s="2" t="n"/>
       <c r="V98" s="2" t="n"/>
-      <c r="W98" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="W98" s="2" t="n"/>
       <c r="X98" s="2" t="n"/>
     </row>
     <row r="99" ht="30" customHeight="1">

</xml_diff>